<commit_message>
update import fields in transactions
</commit_message>
<xml_diff>
--- a/static/templates/transactions.xlsx
+++ b/static/templates/transactions.xlsx
@@ -31,6 +31,9 @@
     <t>Category Name</t>
   </si>
   <si>
+    <t>Source of Funds</t>
+  </si>
+  <si>
     <t>2026-07-15</t>
   </si>
   <si>
@@ -41,6 +44,9 @@
   </si>
   <si>
     <t>Salary</t>
+  </si>
+  <si>
+    <t>Bank Transfer</t>
   </si>
 </sst>
 </file>
@@ -79,6 +85,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -96,22 +110,28 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>50000</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>